<commit_message>
fix tabtools: standardize table rendering across sinks
Prevent published outputs from losing headers, annotations, or formatting when
different tabtools sinks render the same table. Version 1.11.0 fixes regtab
multi-model factor handling, Excel merging, and confidence-limit width; aligns
table1_tc descriptors, Markdown headers, stacktab columnmerge() headers,
generated legends, rate CI separators, negative-zero handling, p-value
phrasing, and footnote punctuation. Make _tabtools_markdown_write.ado require
explicit title() and quiet _tabtools_csv_write.ado internal export chatter.
Bump tabtools to 1.11.0, sync .ado, .pkg, .sthlp, and README files, and
regenerate the checked-in demo workbooks and demo_markdown_report.md.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_corrtab.xlsx
+++ b/tabtools/demo/demo_corrtab.xlsx
@@ -38,7 +38,7 @@
     <t>-0.01</t>
   </si>
   <si>
-    <t>-0.00</t>
+    <t>0.00</t>
   </si>
   <si>
     <t>0.01</t>
@@ -50,10 +50,10 @@
     <t>Table 14. Spearman Rank Correlation Matrix</t>
   </si>
   <si>
-    <t>-0.00 (0.616)</t>
+    <t>0.00 (0.616)</t>
   </si>
   <si>
-    <t>-0.00 (0.807)</t>
+    <t>0.00 (0.807)</t>
   </si>
   <si>
     <t>0.01 (0.450)</t>

</xml_diff>